<commit_message>
Update data laporan bulan Juli 2026
</commit_message>
<xml_diff>
--- a/data/laporan_keuangan.xlsx
+++ b/data/laporan_keuangan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sandaranggas/Library/CloudStorage/GoogleDrive-admin@sandarangga.com/My Drive/Pribadi (1)/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB90E2D1-B951-0442-AE68-A87AF692E558}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DF47169-80B4-7A45-812E-74E4032F56A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17480" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -95,7 +95,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="949" uniqueCount="710">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="955" uniqueCount="713">
   <si>
     <t>NO</t>
   </si>
@@ -2225,6 +2225,15 @@
   </si>
   <si>
     <t>Penghitungan Kotak Amal 14 Juni 2026</t>
+  </si>
+  <si>
+    <t>Gaji Bang Zaini Bulan Juni</t>
+  </si>
+  <si>
+    <t>infaq khotib jum'at</t>
+  </si>
+  <si>
+    <t>Token Listrik 500 Ribu</t>
   </si>
 </sst>
 </file>
@@ -2999,10 +3008,10 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -17627,9 +17636,6 @@
         <f t="shared" si="21"/>
         <v>9228600</v>
       </c>
-      <c r="H629">
-        <v>1446000</v>
-      </c>
     </row>
     <row r="630" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A630" s="19">
@@ -17649,9 +17655,6 @@
         <f t="shared" si="21"/>
         <v>9028600</v>
       </c>
-      <c r="H630">
-        <v>800000</v>
-      </c>
     </row>
     <row r="631" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A631" s="19">
@@ -17671,10 +17674,7 @@
         <f t="shared" si="21"/>
         <v>6968600</v>
       </c>
-      <c r="H631" s="67">
-        <f>H629-H630</f>
-        <v>646000</v>
-      </c>
+      <c r="H631" s="67"/>
     </row>
     <row r="632" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A632" s="19">
@@ -17693,9 +17693,6 @@
       <c r="F632" s="32">
         <f t="shared" si="21"/>
         <v>6818600</v>
-      </c>
-      <c r="H632">
-        <v>500000</v>
       </c>
     </row>
     <row r="633" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -17716,10 +17713,7 @@
         <f t="shared" si="21"/>
         <v>7318600</v>
       </c>
-      <c r="H633" s="67">
-        <f>H631-H632</f>
-        <v>146000</v>
-      </c>
+      <c r="H633" s="67"/>
     </row>
     <row r="634" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A634" s="19">
@@ -18080,7 +18074,7 @@
       </c>
       <c r="E652" s="37"/>
       <c r="F652" s="79">
-        <f t="shared" ref="F652:F684" si="23">F651+D652-E652</f>
+        <f t="shared" ref="F652:F690" si="23">F651+D652-E652</f>
         <v>8218600</v>
       </c>
     </row>
@@ -18698,161 +18692,232 @@
       <c r="A685" s="19">
         <v>633</v>
       </c>
-      <c r="B685" s="68"/>
-      <c r="C685" s="36"/>
+      <c r="B685" s="68">
+        <v>46198</v>
+      </c>
+      <c r="C685" s="36" t="s">
+        <v>710</v>
+      </c>
       <c r="D685" s="37"/>
-      <c r="E685" s="37"/>
-      <c r="F685" s="79"/>
+      <c r="E685" s="37">
+        <v>600000</v>
+      </c>
+      <c r="F685" s="79">
+        <f t="shared" si="23"/>
+        <v>17442601</v>
+      </c>
     </row>
     <row r="686" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A686" s="19">
         <v>634</v>
       </c>
-      <c r="B686" s="68"/>
-      <c r="C686" s="36"/>
+      <c r="B686" s="68">
+        <v>46199</v>
+      </c>
+      <c r="C686" s="36" t="s">
+        <v>711</v>
+      </c>
       <c r="D686" s="37"/>
-      <c r="E686" s="37"/>
-      <c r="F686" s="79"/>
+      <c r="E686" s="37">
+        <v>500000</v>
+      </c>
+      <c r="F686" s="79">
+        <f t="shared" si="23"/>
+        <v>16942601</v>
+      </c>
     </row>
     <row r="687" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A687" s="19"/>
-      <c r="B687" s="81"/>
-      <c r="C687" s="80" t="s">
+      <c r="A687" s="19">
+        <v>635</v>
+      </c>
+      <c r="B687" s="68">
+        <v>46204</v>
+      </c>
+      <c r="C687" s="36" t="s">
+        <v>712</v>
+      </c>
+      <c r="D687" s="37"/>
+      <c r="E687" s="37">
+        <v>500000</v>
+      </c>
+      <c r="F687" s="79">
+        <f t="shared" si="23"/>
+        <v>16442601</v>
+      </c>
+    </row>
+    <row r="688" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A688" s="19">
+        <v>636</v>
+      </c>
+      <c r="B688" s="68">
+        <v>46213</v>
+      </c>
+      <c r="C688" s="36" t="s">
+        <v>712</v>
+      </c>
+      <c r="D688" s="37"/>
+      <c r="E688" s="37">
+        <v>500000</v>
+      </c>
+      <c r="F688" s="79">
+        <f t="shared" si="23"/>
+        <v>15942601</v>
+      </c>
+    </row>
+    <row r="689" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A689" s="19">
+        <v>637</v>
+      </c>
+      <c r="B689" s="68">
+        <v>46220</v>
+      </c>
+      <c r="C689" s="36" t="s">
+        <v>426</v>
+      </c>
+      <c r="D689" s="37"/>
+      <c r="E689" s="37">
+        <v>500000</v>
+      </c>
+      <c r="F689" s="79">
+        <f t="shared" si="23"/>
+        <v>15442601</v>
+      </c>
+      <c r="H689" s="67"/>
+    </row>
+    <row r="690" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A690" s="19">
+        <v>638</v>
+      </c>
+      <c r="B690" s="68">
+        <v>46221</v>
+      </c>
+      <c r="C690" s="36" t="s">
+        <v>708</v>
+      </c>
+      <c r="D690" s="37">
+        <v>300000</v>
+      </c>
+      <c r="E690" s="37"/>
+      <c r="F690" s="79">
+        <f t="shared" si="23"/>
+        <v>15742601</v>
+      </c>
+    </row>
+    <row r="691" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A691" s="19">
+        <v>639</v>
+      </c>
+      <c r="B691" s="68"/>
+      <c r="C691" s="36"/>
+      <c r="D691" s="37"/>
+      <c r="E691" s="37"/>
+      <c r="F691" s="79"/>
+    </row>
+    <row r="692" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A692" s="19">
+        <v>640</v>
+      </c>
+      <c r="B692" s="68"/>
+      <c r="C692" s="36"/>
+      <c r="D692" s="37"/>
+      <c r="E692" s="37"/>
+      <c r="F692" s="79"/>
+    </row>
+    <row r="693" spans="1:8" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A693" s="19"/>
+      <c r="B693" s="81"/>
+      <c r="C693" s="80" t="s">
         <v>191</v>
       </c>
-      <c r="D687" s="74"/>
-      <c r="E687" s="74"/>
-      <c r="F687" s="78">
-        <f>F684</f>
-        <v>18042601</v>
-      </c>
-    </row>
-    <row r="688" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B688" s="1"/>
-      <c r="C688" s="1"/>
-      <c r="D688" s="1"/>
-      <c r="E688" s="1"/>
-      <c r="F688" s="1"/>
-    </row>
-    <row r="689" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B689" s="1"/>
-      <c r="C689" s="1"/>
-      <c r="D689" s="1"/>
-      <c r="E689" s="23" t="s">
-        <v>656</v>
-      </c>
-    </row>
-    <row r="690" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B690" s="91" t="s">
-        <v>192</v>
-      </c>
-      <c r="C690" s="89"/>
-      <c r="D690" s="1"/>
-      <c r="E690" s="1"/>
-      <c r="F690" s="1"/>
-    </row>
-    <row r="691" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B691" s="23"/>
-      <c r="C691" s="1"/>
-      <c r="D691" s="1"/>
-    </row>
-    <row r="692" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B692" s="22" t="s">
-        <v>193</v>
-      </c>
-      <c r="C692" s="1"/>
-      <c r="D692" s="1"/>
-      <c r="E692" s="23" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="693" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B693" s="23"/>
-      <c r="C693" s="1"/>
-      <c r="D693" s="1"/>
-      <c r="E693" s="1"/>
-      <c r="F693" s="1"/>
-    </row>
-    <row r="694" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D693" s="74"/>
+      <c r="E693" s="74"/>
+      <c r="F693" s="78">
+        <f>F690</f>
+        <v>15742601</v>
+      </c>
+    </row>
+    <row r="694" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B694" s="1"/>
       <c r="C694" s="1"/>
       <c r="D694" s="1"/>
       <c r="E694" s="1"/>
       <c r="F694" s="1"/>
     </row>
-    <row r="695" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B695" s="1" t="s">
-        <v>195</v>
-      </c>
+    <row r="695" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B695" s="1"/>
       <c r="C695" s="1"/>
       <c r="D695" s="1"/>
       <c r="E695" s="23" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="696" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B696" s="1"/>
-      <c r="C696" s="1"/>
+        <v>656</v>
+      </c>
+    </row>
+    <row r="696" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B696" s="91" t="s">
+        <v>192</v>
+      </c>
+      <c r="C696" s="89"/>
       <c r="D696" s="1"/>
       <c r="E696" s="1"/>
       <c r="F696" s="1"/>
     </row>
-    <row r="697" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="697" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B697" s="23"/>
       <c r="C697" s="1"/>
       <c r="D697" s="1"/>
-      <c r="E697">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="698" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B698" s="1"/>
+    </row>
+    <row r="698" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B698" s="22" t="s">
+        <v>193</v>
+      </c>
       <c r="C698" s="1"/>
       <c r="D698" s="1"/>
-    </row>
-    <row r="699" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B699" s="1"/>
+      <c r="E698" s="23" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="699" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B699" s="23"/>
       <c r="C699" s="1"/>
       <c r="D699" s="1"/>
       <c r="E699" s="1"/>
       <c r="F699" s="1"/>
     </row>
-    <row r="700" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="700" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B700" s="1"/>
       <c r="C700" s="1"/>
       <c r="D700" s="1"/>
       <c r="E700" s="1"/>
       <c r="F700" s="1"/>
     </row>
-    <row r="701" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B701" s="24" t="s">
-        <v>197</v>
+    <row r="701" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B701" s="1" t="s">
+        <v>195</v>
       </c>
       <c r="C701" s="1"/>
       <c r="D701" s="1"/>
-      <c r="E701" s="1"/>
-      <c r="F701" s="1"/>
-    </row>
-    <row r="702" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E701" s="23" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="702" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B702" s="1"/>
       <c r="C702" s="1"/>
       <c r="D702" s="1"/>
       <c r="E702" s="1"/>
       <c r="F702" s="1"/>
     </row>
-    <row r="703" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B703" s="1"/>
+    <row r="703" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B703" s="23"/>
       <c r="C703" s="1"/>
       <c r="D703" s="1"/>
-      <c r="E703" s="1"/>
-      <c r="F703" s="1"/>
-    </row>
-    <row r="704" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E703">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="704" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B704" s="1"/>
       <c r="C704" s="1"/>
       <c r="D704" s="1"/>
-      <c r="E704" s="1"/>
-      <c r="F704" s="1"/>
     </row>
     <row r="705" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B705" s="1"/>
@@ -18869,7 +18934,9 @@
       <c r="F706" s="1"/>
     </row>
     <row r="707" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B707" s="1"/>
+      <c r="B707" s="24" t="s">
+        <v>197</v>
+      </c>
       <c r="C707" s="1"/>
       <c r="D707" s="1"/>
       <c r="E707" s="1"/>
@@ -19218,12 +19285,48 @@
       <c r="E756" s="1"/>
       <c r="F756" s="1"/>
     </row>
-    <row r="757" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="758" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="759" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="760" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="761" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="762" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="757" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B757" s="1"/>
+      <c r="C757" s="1"/>
+      <c r="D757" s="1"/>
+      <c r="E757" s="1"/>
+      <c r="F757" s="1"/>
+    </row>
+    <row r="758" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B758" s="1"/>
+      <c r="C758" s="1"/>
+      <c r="D758" s="1"/>
+      <c r="E758" s="1"/>
+      <c r="F758" s="1"/>
+    </row>
+    <row r="759" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B759" s="1"/>
+      <c r="C759" s="1"/>
+      <c r="D759" s="1"/>
+      <c r="E759" s="1"/>
+      <c r="F759" s="1"/>
+    </row>
+    <row r="760" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B760" s="1"/>
+      <c r="C760" s="1"/>
+      <c r="D760" s="1"/>
+      <c r="E760" s="1"/>
+      <c r="F760" s="1"/>
+    </row>
+    <row r="761" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B761" s="1"/>
+      <c r="C761" s="1"/>
+      <c r="D761" s="1"/>
+      <c r="E761" s="1"/>
+      <c r="F761" s="1"/>
+    </row>
+    <row r="762" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B762" s="1"/>
+      <c r="C762" s="1"/>
+      <c r="D762" s="1"/>
+      <c r="E762" s="1"/>
+      <c r="F762" s="1"/>
+    </row>
     <row r="763" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="764" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="765" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -19487,10 +19590,10 @@
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="B690:C690"/>
+    <mergeCell ref="B696:C696"/>
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
-  <conditionalFormatting sqref="B134:B686">
+  <conditionalFormatting sqref="B134:B692">
     <cfRule type="timePeriod" dxfId="5" priority="3" timePeriod="today">
       <formula>FLOOR(B134,1)=TODAY()</formula>
     </cfRule>
@@ -19526,11 +19629,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="87" t="s">
+      <c r="A1" s="86" t="s">
         <v>460</v>
       </c>
-      <c r="B1" s="87"/>
-      <c r="C1" s="87"/>
+      <c r="B1" s="86"/>
+      <c r="C1" s="86"/>
     </row>
     <row r="2" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2">
@@ -19702,11 +19805,11 @@
       </c>
     </row>
     <row r="18" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="87" t="s">
+      <c r="A18" s="86" t="s">
         <v>486</v>
       </c>
-      <c r="B18" s="87"/>
-      <c r="C18" s="87"/>
+      <c r="B18" s="86"/>
+      <c r="C18" s="86"/>
     </row>
     <row r="19" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="48">
@@ -19751,11 +19854,11 @@
       </c>
     </row>
     <row r="23" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="87" t="s">
+      <c r="A23" s="86" t="s">
         <v>498</v>
       </c>
-      <c r="B23" s="87"/>
-      <c r="C23" s="87"/>
+      <c r="B23" s="86"/>
+      <c r="C23" s="86"/>
     </row>
     <row r="24" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="48">
@@ -19849,11 +19952,11 @@
     </row>
     <row r="32" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="33" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="87" t="s">
+      <c r="A33" s="86" t="s">
         <v>499</v>
       </c>
-      <c r="B33" s="87"/>
-      <c r="C33" s="87"/>
+      <c r="B33" s="86"/>
+      <c r="C33" s="86"/>
     </row>
     <row r="34" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="48">
@@ -19946,11 +20049,11 @@
       </c>
     </row>
     <row r="42" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="87" t="s">
+      <c r="A42" s="86" t="s">
         <v>504</v>
       </c>
-      <c r="B42" s="87"/>
-      <c r="C42" s="87"/>
+      <c r="B42" s="86"/>
+      <c r="C42" s="86"/>
     </row>
     <row r="43" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="48">
@@ -20044,11 +20147,11 @@
     </row>
     <row r="51" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="52" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="87" t="s">
+      <c r="A52" s="86" t="s">
         <v>507</v>
       </c>
-      <c r="B52" s="87"/>
-      <c r="C52" s="87"/>
+      <c r="B52" s="86"/>
+      <c r="C52" s="86"/>
     </row>
     <row r="53" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="48">
@@ -20142,11 +20245,11 @@
     </row>
     <row r="61" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="62" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="87" t="s">
+      <c r="A62" s="86" t="s">
         <v>513</v>
       </c>
-      <c r="B62" s="87"/>
-      <c r="C62" s="87"/>
+      <c r="B62" s="86"/>
+      <c r="C62" s="86"/>
     </row>
     <row r="63" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="48">
@@ -20241,11 +20344,11 @@
     <row r="71" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="72" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="73" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A73" s="87" t="s">
+      <c r="A73" s="86" t="s">
         <v>526</v>
       </c>
-      <c r="B73" s="87"/>
-      <c r="C73" s="87"/>
+      <c r="B73" s="86"/>
+      <c r="C73" s="86"/>
     </row>
     <row r="74" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="48">
@@ -20352,11 +20455,11 @@
     <row r="83" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="84" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="85" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A85" s="87" t="s">
+      <c r="A85" s="86" t="s">
         <v>535</v>
       </c>
-      <c r="B85" s="87"/>
-      <c r="C85" s="87"/>
+      <c r="B85" s="86"/>
+      <c r="C85" s="86"/>
     </row>
     <row r="86" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="48">
@@ -20446,11 +20549,11 @@
     </row>
     <row r="95" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="96" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A96" s="87" t="s">
+      <c r="A96" s="86" t="s">
         <v>541</v>
       </c>
-      <c r="B96" s="87"/>
-      <c r="C96" s="87"/>
+      <c r="B96" s="86"/>
+      <c r="C96" s="86"/>
     </row>
     <row r="97" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="48">
@@ -20548,11 +20651,11 @@
     </row>
     <row r="106" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="107" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A107" s="87" t="s">
+      <c r="A107" s="86" t="s">
         <v>542</v>
       </c>
-      <c r="B107" s="87"/>
-      <c r="C107" s="87"/>
+      <c r="B107" s="86"/>
+      <c r="C107" s="86"/>
     </row>
     <row r="108" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="48">
@@ -20650,11 +20753,11 @@
     </row>
     <row r="117" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="118" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A118" s="87" t="s">
+      <c r="A118" s="86" t="s">
         <v>543</v>
       </c>
-      <c r="B118" s="87"/>
-      <c r="C118" s="87"/>
+      <c r="B118" s="86"/>
+      <c r="C118" s="86"/>
     </row>
     <row r="119" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="48">
@@ -20752,11 +20855,11 @@
     </row>
     <row r="128" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="129" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A129" s="86" t="s">
+      <c r="A129" s="87" t="s">
         <v>555</v>
       </c>
-      <c r="B129" s="87"/>
-      <c r="C129" s="87"/>
+      <c r="B129" s="86"/>
+      <c r="C129" s="86"/>
     </row>
     <row r="130" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" s="48">
@@ -20854,11 +20957,11 @@
     </row>
     <row r="139" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="140" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A140" s="86" t="s">
+      <c r="A140" s="87" t="s">
         <v>556</v>
       </c>
-      <c r="B140" s="87"/>
-      <c r="C140" s="87"/>
+      <c r="B140" s="86"/>
+      <c r="C140" s="86"/>
     </row>
     <row r="141" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141" s="48">
@@ -20956,11 +21059,11 @@
     </row>
     <row r="150" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="151" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A151" s="86" t="s">
+      <c r="A151" s="87" t="s">
         <v>562</v>
       </c>
-      <c r="B151" s="87"/>
-      <c r="C151" s="87"/>
+      <c r="B151" s="86"/>
+      <c r="C151" s="86"/>
     </row>
     <row r="152" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A152" s="48">
@@ -21058,11 +21161,11 @@
     </row>
     <row r="161" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="162" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A162" s="86" t="s">
+      <c r="A162" s="87" t="s">
         <v>572</v>
       </c>
-      <c r="B162" s="87"/>
-      <c r="C162" s="87"/>
+      <c r="B162" s="86"/>
+      <c r="C162" s="86"/>
     </row>
     <row r="163" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A163" s="48">
@@ -21160,11 +21263,11 @@
     </row>
     <row r="172" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="173" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A173" s="86" t="s">
+      <c r="A173" s="87" t="s">
         <v>573</v>
       </c>
-      <c r="B173" s="87"/>
-      <c r="C173" s="87"/>
+      <c r="B173" s="86"/>
+      <c r="C173" s="86"/>
     </row>
     <row r="174" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A174" s="48">
@@ -23404,20 +23507,6 @@
     <row r="1000" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="A275:C275"/>
-    <mergeCell ref="A228:C228"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="A42:C42"/>
-    <mergeCell ref="A73:C73"/>
-    <mergeCell ref="A52:C52"/>
-    <mergeCell ref="A62:C62"/>
-    <mergeCell ref="A107:C107"/>
-    <mergeCell ref="A118:C118"/>
-    <mergeCell ref="A96:C96"/>
-    <mergeCell ref="A85:C85"/>
     <mergeCell ref="A333:C333"/>
     <mergeCell ref="A173:C173"/>
     <mergeCell ref="A151:C151"/>
@@ -23434,6 +23523,20 @@
     <mergeCell ref="A206:C206"/>
     <mergeCell ref="A309:C309"/>
     <mergeCell ref="A286:C286"/>
+    <mergeCell ref="A275:C275"/>
+    <mergeCell ref="A228:C228"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="A73:C73"/>
+    <mergeCell ref="A52:C52"/>
+    <mergeCell ref="A62:C62"/>
+    <mergeCell ref="A107:C107"/>
+    <mergeCell ref="A118:C118"/>
+    <mergeCell ref="A96:C96"/>
+    <mergeCell ref="A85:C85"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>

<commit_message>
Update ledger via dashboard admin
</commit_message>
<xml_diff>
--- a/data/laporan_keuangan.xlsx
+++ b/data/laporan_keuangan.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G685"/>
+  <dimension ref="A1:G686"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -12236,56 +12236,56 @@
     </row>
     <row r="438">
       <c r="A438" t="n">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B438" s="2" t="n">
         <v>45353</v>
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>Sumbangan Hamba Allah</t>
+          <t>Infaq untuk Ustadz Tarhib Ramadhan</t>
         </is>
       </c>
       <c r="D438" t="inlineStr">
         <is>
-          <t>Infaq &amp; Sumbangan Lain</t>
+          <t>Infaq Ustadz/Khotib/Imam</t>
         </is>
       </c>
       <c r="E438" s="3" t="n">
-        <v>5000000</v>
+        <v>0</v>
       </c>
       <c r="F438" s="3" t="n">
-        <v>0</v>
+        <v>1500000</v>
       </c>
       <c r="G438" s="3" t="n">
-        <v>5119290</v>
+        <v>3619290</v>
       </c>
     </row>
     <row r="439">
       <c r="A439" t="n">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="B439" s="2" t="n">
         <v>45353</v>
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>Infaq untuk Ustadz Tarhib Ramadhan</t>
+          <t>Sumbangan Hamba Allah</t>
         </is>
       </c>
       <c r="D439" t="inlineStr">
         <is>
-          <t>Infaq Ustadz/Khotib/Imam</t>
+          <t>Infaq &amp; Sumbangan Lain</t>
         </is>
       </c>
       <c r="E439" s="3" t="n">
-        <v>0</v>
+        <v>5000000</v>
       </c>
       <c r="F439" s="3" t="n">
-        <v>1500000</v>
+        <v>0</v>
       </c>
       <c r="G439" s="3" t="n">
-        <v>3619290</v>
+        <v>5119290</v>
       </c>
     </row>
     <row r="440">
@@ -15125,56 +15125,56 @@
     </row>
     <row r="545">
       <c r="A545" t="n">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B545" s="2" t="n">
         <v>45773</v>
       </c>
       <c r="C545" t="inlineStr">
         <is>
-          <t>Reimburse Infaq Khotib Jum'at 25 April 2025</t>
+          <t>Pembelian Token Listrik</t>
         </is>
       </c>
       <c r="D545" t="inlineStr">
         <is>
-          <t>Infaq Ustadz/Khotib/Imam</t>
+          <t>Listrik &amp; Perawatan</t>
         </is>
       </c>
       <c r="E545" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F545" s="3" t="n">
-        <v>500000</v>
+        <v>1000000</v>
       </c>
       <c r="G545" s="3" t="n">
-        <v>5223000</v>
+        <v>4223000</v>
       </c>
     </row>
     <row r="546">
       <c r="A546" t="n">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="B546" s="2" t="n">
         <v>45773</v>
       </c>
       <c r="C546" t="inlineStr">
         <is>
-          <t>Pembelian Token Listrik</t>
+          <t>Reimburse Infaq Khotib Jum'at 25 April 2025</t>
         </is>
       </c>
       <c r="D546" t="inlineStr">
         <is>
-          <t>Listrik &amp; Perawatan</t>
+          <t>Infaq Ustadz/Khotib/Imam</t>
         </is>
       </c>
       <c r="E546" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F546" s="3" t="n">
-        <v>1000000</v>
+        <v>500000</v>
       </c>
       <c r="G546" s="3" t="n">
-        <v>4223000</v>
+        <v>5223000</v>
       </c>
     </row>
     <row r="547">
@@ -15422,56 +15422,56 @@
     </row>
     <row r="556">
       <c r="A556" t="n">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B556" s="2" t="n">
         <v>45802</v>
       </c>
       <c r="C556" t="inlineStr">
         <is>
-          <t>Gaji Bang Zaeni Bulan Mei</t>
+          <t>infaq dari Jamaah via transfer dan QRIS</t>
         </is>
       </c>
       <c r="D556" t="inlineStr">
         <is>
-          <t>Gaji Marbot / Staf</t>
+          <t>Infaq Rekening/QRIS</t>
         </is>
       </c>
       <c r="E556" s="3" t="n">
-        <v>0</v>
+        <v>1370500</v>
       </c>
       <c r="F556" s="3" t="n">
-        <v>600000</v>
+        <v>0</v>
       </c>
       <c r="G556" s="3" t="n">
-        <v>6577600</v>
+        <v>7948100</v>
       </c>
     </row>
     <row r="557">
       <c r="A557" t="n">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="B557" s="2" t="n">
         <v>45802</v>
       </c>
       <c r="C557" t="inlineStr">
         <is>
-          <t>infaq dari Jamaah via transfer dan QRIS</t>
+          <t>Gaji Bang Zaeni Bulan Mei</t>
         </is>
       </c>
       <c r="D557" t="inlineStr">
         <is>
-          <t>Infaq Rekening/QRIS</t>
+          <t>Gaji Marbot / Staf</t>
         </is>
       </c>
       <c r="E557" s="3" t="n">
-        <v>1370500</v>
+        <v>0</v>
       </c>
       <c r="F557" s="3" t="n">
-        <v>0</v>
+        <v>600000</v>
       </c>
       <c r="G557" s="3" t="n">
-        <v>7948100</v>
+        <v>6577600</v>
       </c>
     </row>
     <row r="558">
@@ -15719,83 +15719,83 @@
     </row>
     <row r="567">
       <c r="A567" t="n">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="B567" s="2" t="n">
         <v>45838</v>
       </c>
       <c r="C567" t="inlineStr">
         <is>
-          <t>Subsidi TPA Bulan Juni 2025</t>
+          <t>infaq dari Jamaah via transfer dan QRIS</t>
         </is>
       </c>
       <c r="D567" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>Infaq Rekening/QRIS</t>
         </is>
       </c>
       <c r="E567" s="3" t="n">
-        <v>0</v>
+        <v>255000</v>
       </c>
       <c r="F567" s="3" t="n">
-        <v>1200000</v>
+        <v>0</v>
       </c>
       <c r="G567" s="3" t="n">
-        <v>4540100</v>
+        <v>6656100</v>
       </c>
     </row>
     <row r="568">
       <c r="A568" t="n">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B568" s="2" t="n">
         <v>45838</v>
       </c>
       <c r="C568" t="inlineStr">
         <is>
-          <t>Setoran Pembukaan Kotak Amal 30 Juni 2025</t>
+          <t>Subsidi TPA Bulan Juni 2025</t>
         </is>
       </c>
       <c r="D568" t="inlineStr">
         <is>
-          <t>Kotak Amal / Kencleng</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="E568" s="3" t="n">
-        <v>1861000</v>
+        <v>0</v>
       </c>
       <c r="F568" s="3" t="n">
-        <v>0</v>
+        <v>1200000</v>
       </c>
       <c r="G568" s="3" t="n">
-        <v>6401100</v>
+        <v>4540100</v>
       </c>
     </row>
     <row r="569">
       <c r="A569" t="n">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="B569" s="2" t="n">
         <v>45838</v>
       </c>
       <c r="C569" t="inlineStr">
         <is>
-          <t>infaq dari Jamaah via transfer dan QRIS</t>
+          <t>Setoran Pembukaan Kotak Amal 30 Juni 2025</t>
         </is>
       </c>
       <c r="D569" t="inlineStr">
         <is>
-          <t>Infaq Rekening/QRIS</t>
+          <t>Kotak Amal / Kencleng</t>
         </is>
       </c>
       <c r="E569" s="3" t="n">
-        <v>255000</v>
+        <v>1861000</v>
       </c>
       <c r="F569" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G569" s="3" t="n">
-        <v>6656100</v>
+        <v>6401100</v>
       </c>
     </row>
     <row r="570">
@@ -17312,41 +17312,41 @@
     </row>
     <row r="626">
       <c r="A626" t="n">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="B626" s="2" t="n">
         <v>46053</v>
       </c>
       <c r="C626" t="inlineStr">
         <is>
-          <t>Realisasi Pengajuan Majelis Ta'lim</t>
+          <t>Rekapan Infaq di rekening / QRIS</t>
         </is>
       </c>
       <c r="D626" t="inlineStr">
         <is>
-          <t>Majelis Ta'lim</t>
+          <t>Infaq Rekening/QRIS</t>
         </is>
       </c>
       <c r="E626" s="3" t="n">
-        <v>0</v>
+        <v>300000</v>
       </c>
       <c r="F626" s="3" t="n">
-        <v>500000</v>
+        <v>0</v>
       </c>
       <c r="G626" s="3" t="n">
-        <v>5618600</v>
+        <v>5918600</v>
       </c>
     </row>
     <row r="627">
       <c r="A627" t="n">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="B627" s="2" t="n">
         <v>46053</v>
       </c>
       <c r="C627" t="inlineStr">
         <is>
-          <t>Dana Kegiatan TPA Al Ikhlas</t>
+          <t>Subsidi TPA Bulan Januari 2026</t>
         </is>
       </c>
       <c r="D627" t="inlineStr">
@@ -17361,61 +17361,61 @@
         <v>1200000</v>
       </c>
       <c r="G627" s="3" t="n">
-        <v>6118600</v>
+        <v>4718600</v>
       </c>
     </row>
     <row r="628">
       <c r="A628" t="n">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="B628" s="2" t="n">
         <v>46053</v>
       </c>
       <c r="C628" t="inlineStr">
         <is>
-          <t>Rekapan Infaq di rekening / QRIS</t>
+          <t>Dana Kegiatan TPA Al Ikhlas</t>
         </is>
       </c>
       <c r="D628" t="inlineStr">
         <is>
-          <t>Infaq Rekening/QRIS</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="E628" s="3" t="n">
-        <v>300000</v>
+        <v>0</v>
       </c>
       <c r="F628" s="3" t="n">
-        <v>0</v>
+        <v>1200000</v>
       </c>
       <c r="G628" s="3" t="n">
-        <v>5918600</v>
+        <v>6118600</v>
       </c>
     </row>
     <row r="629">
       <c r="A629" t="n">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="B629" s="2" t="n">
         <v>46053</v>
       </c>
       <c r="C629" t="inlineStr">
         <is>
-          <t>Subsidi TPA Bulan Januari 2026</t>
+          <t>Realisasi Pengajuan Majelis Ta'lim</t>
         </is>
       </c>
       <c r="D629" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>Majelis Ta'lim</t>
         </is>
       </c>
       <c r="E629" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F629" s="3" t="n">
-        <v>1200000</v>
+        <v>500000</v>
       </c>
       <c r="G629" s="3" t="n">
-        <v>4718600</v>
+        <v>5618600</v>
       </c>
     </row>
     <row r="630">
@@ -17663,56 +17663,56 @@
     </row>
     <row r="639">
       <c r="A639" t="n">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B639" s="2" t="n">
         <v>46074</v>
       </c>
       <c r="C639" t="inlineStr">
         <is>
-          <t>Sumbangan Kantor Pak Jalal</t>
+          <t>Infaq Imam dan Ceramah Tarawih</t>
         </is>
       </c>
       <c r="D639" t="inlineStr">
         <is>
-          <t>Infaq &amp; Sumbangan Lain</t>
+          <t>Infaq Ustadz/Khotib/Imam</t>
         </is>
       </c>
       <c r="E639" s="3" t="n">
-        <v>10000000</v>
+        <v>0</v>
       </c>
       <c r="F639" s="3" t="n">
-        <v>0</v>
+        <v>1500000</v>
       </c>
       <c r="G639" s="3" t="n">
-        <v>11318600</v>
+        <v>9818600</v>
       </c>
     </row>
     <row r="640">
       <c r="A640" t="n">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B640" s="2" t="n">
         <v>46074</v>
       </c>
       <c r="C640" t="inlineStr">
         <is>
-          <t>Infaq Imam dan Ceramah Tarawih</t>
+          <t>Sumbangan Kantor Pak Jalal</t>
         </is>
       </c>
       <c r="D640" t="inlineStr">
         <is>
-          <t>Infaq Ustadz/Khotib/Imam</t>
+          <t>Infaq &amp; Sumbangan Lain</t>
         </is>
       </c>
       <c r="E640" s="3" t="n">
-        <v>0</v>
+        <v>10000000</v>
       </c>
       <c r="F640" s="3" t="n">
-        <v>1500000</v>
+        <v>0</v>
       </c>
       <c r="G640" s="3" t="n">
-        <v>9818600</v>
+        <v>11318600</v>
       </c>
     </row>
     <row r="641">
@@ -17987,56 +17987,56 @@
     </row>
     <row r="651">
       <c r="A651" t="n">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="B651" s="2" t="n">
         <v>46094</v>
       </c>
       <c r="C651" t="inlineStr">
         <is>
-          <t>Subsidi TPA Bulan Maret 2026</t>
+          <t>Rekapan Infaq di rekening / QRIS per 13 Maret 2026</t>
         </is>
       </c>
       <c r="D651" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>Infaq Rekening/QRIS</t>
         </is>
       </c>
       <c r="E651" s="3" t="n">
-        <v>0</v>
+        <v>1982000</v>
       </c>
       <c r="F651" s="3" t="n">
-        <v>1100000</v>
+        <v>0</v>
       </c>
       <c r="G651" s="3" t="n">
-        <v>8896600</v>
+        <v>10878600</v>
       </c>
     </row>
     <row r="652">
       <c r="A652" t="n">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B652" s="2" t="n">
         <v>46094</v>
       </c>
       <c r="C652" t="inlineStr">
         <is>
-          <t>Rekapan Infaq di rekening / QRIS per 13 Maret 2026</t>
+          <t>Subsidi TPA Bulan Maret 2026</t>
         </is>
       </c>
       <c r="D652" t="inlineStr">
         <is>
-          <t>Infaq Rekening/QRIS</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="E652" s="3" t="n">
-        <v>1982000</v>
+        <v>0</v>
       </c>
       <c r="F652" s="3" t="n">
-        <v>0</v>
+        <v>1100000</v>
       </c>
       <c r="G652" s="3" t="n">
-        <v>10878600</v>
+        <v>8896600</v>
       </c>
     </row>
     <row r="653">
@@ -18284,56 +18284,56 @@
     </row>
     <row r="662">
       <c r="A662" t="n">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="B662" s="2" t="n">
         <v>46137</v>
       </c>
       <c r="C662" t="inlineStr">
         <is>
-          <t>Infaq Khotib Jum'at</t>
+          <t>Gaji Bang Zaeini Bulan April</t>
         </is>
       </c>
       <c r="D662" t="inlineStr">
         <is>
-          <t>Infaq Ustadz/Khotib/Imam</t>
+          <t>Gaji Marbot / Staf</t>
         </is>
       </c>
       <c r="E662" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F662" s="3" t="n">
-        <v>500000</v>
+        <v>600000</v>
       </c>
       <c r="G662" s="3" t="n">
-        <v>10191600</v>
+        <v>9591600</v>
       </c>
     </row>
     <row r="663">
       <c r="A663" t="n">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="B663" s="2" t="n">
         <v>46137</v>
       </c>
       <c r="C663" t="inlineStr">
         <is>
-          <t>Gaji Bang Zaeini Bulan April</t>
+          <t>Infaq Khotib Jum'at</t>
         </is>
       </c>
       <c r="D663" t="inlineStr">
         <is>
-          <t>Gaji Marbot / Staf</t>
+          <t>Infaq Ustadz/Khotib/Imam</t>
         </is>
       </c>
       <c r="E663" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F663" s="3" t="n">
-        <v>600000</v>
+        <v>500000</v>
       </c>
       <c r="G663" s="3" t="n">
-        <v>9591600</v>
+        <v>10191600</v>
       </c>
     </row>
     <row r="664">
@@ -18500,110 +18500,110 @@
     </row>
     <row r="670">
       <c r="A670" t="n">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="B670" s="2" t="n">
         <v>46172</v>
       </c>
       <c r="C670" t="inlineStr">
         <is>
-          <t>Tambahan Infaq Ustadz untuk acara remaja masjid</t>
+          <t>Subsidi TPA Bulan Mei 2026</t>
         </is>
       </c>
       <c r="D670" t="inlineStr">
         <is>
-          <t>Infaq Ustadz/Khotib/Imam</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="E670" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F670" s="3" t="n">
-        <v>300000</v>
+        <v>800000</v>
       </c>
       <c r="G670" s="3" t="n">
-        <v>7891600</v>
+        <v>7091600</v>
       </c>
     </row>
     <row r="671">
       <c r="A671" t="n">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="B671" s="2" t="n">
         <v>46172</v>
       </c>
       <c r="C671" t="inlineStr">
         <is>
-          <t>Subsidi TPA Bulan Mei 2026</t>
+          <t>Tambahan Infaq Ustadz untuk acara remaja masjid</t>
         </is>
       </c>
       <c r="D671" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>Infaq Ustadz/Khotib/Imam</t>
         </is>
       </c>
       <c r="E671" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F671" s="3" t="n">
-        <v>800000</v>
+        <v>300000</v>
       </c>
       <c r="G671" s="3" t="n">
-        <v>7091600</v>
+        <v>7891600</v>
       </c>
     </row>
     <row r="672">
       <c r="A672" t="n">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="B672" s="2" t="n">
         <v>46173</v>
       </c>
       <c r="C672" t="inlineStr">
         <is>
-          <t>Penghitungan Kotak Amal 21 Mei 2026</t>
+          <t>Rekapan Infaq di rekening / QRIS/</t>
         </is>
       </c>
       <c r="D672" t="inlineStr">
         <is>
-          <t>Kotak Amal / Kencleng</t>
+          <t>Infaq Rekening/QRIS</t>
         </is>
       </c>
       <c r="E672" s="3" t="n">
-        <v>2115000</v>
+        <v>4658001</v>
       </c>
       <c r="F672" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G672" s="3" t="n">
-        <v>9206600</v>
+        <v>13864601</v>
       </c>
     </row>
     <row r="673">
       <c r="A673" t="n">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="B673" s="2" t="n">
         <v>46173</v>
       </c>
       <c r="C673" t="inlineStr">
         <is>
-          <t>Rekapan Infaq di rekening / QRIS/</t>
+          <t>Penghitungan Kotak Amal 21 Mei 2026</t>
         </is>
       </c>
       <c r="D673" t="inlineStr">
         <is>
-          <t>Infaq Rekening/QRIS</t>
+          <t>Kotak Amal / Kencleng</t>
         </is>
       </c>
       <c r="E673" s="3" t="n">
-        <v>4658001</v>
+        <v>2115000</v>
       </c>
       <c r="F673" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G673" s="3" t="n">
-        <v>13864601</v>
+        <v>9206600</v>
       </c>
     </row>
     <row r="674">
@@ -18904,15 +18904,42 @@
       </c>
     </row>
     <row r="685">
-      <c r="C685" s="4" t="inlineStr">
+      <c r="A685" t="n">
+        <v>641</v>
+      </c>
+      <c r="B685" s="2" t="n">
+        <v>46230</v>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>Pemasukan Kotak Amal</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>Kotak Amal / Kencleng</t>
+        </is>
+      </c>
+      <c r="E685" s="3" t="n">
+        <v>3108000</v>
+      </c>
+      <c r="F685" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G685" s="3" t="n">
+        <v>18819934</v>
+      </c>
+    </row>
+    <row r="686">
+      <c r="C686" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E685" s="5" t="n">
-        <v>378166644</v>
-      </c>
-      <c r="F685" s="5" t="n">
+      <c r="E686" s="5" t="n">
+        <v>381274644</v>
+      </c>
+      <c r="F686" s="5" t="n">
         <v>360617210</v>
       </c>
     </row>

</xml_diff>